<commit_message>
Revise File 1 Excel and File 2 Word with complete Braille Indikator I file list and direct Admin link
</commit_message>
<xml_diff>
--- a/FILE_1_SPREADSHEET_AKIP_2025_LOKASI_FILE_LAPTOP.xlsx
+++ b/FILE_1_SPREADSHEET_AKIP_2025_LOKASI_FILE_LAPTOP.xlsx
@@ -618,7 +618,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB1044"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="0"/>
   <cols>
     <col width="3.13" customWidth="1" style="53" min="1" max="1"/>
     <col width="8" customWidth="1" style="53" min="2" max="2"/>
@@ -5818,17 +5818,17 @@
       </c>
       <c r="E94" s="16" t="inlineStr">
         <is>
-          <t>Dokumen Formulir Permohonan &amp; Keberatan Huruf Braille serta Laporan Inovasi Layanan Ramah Disabilitas PPID PKTJ Tegal</t>
+          <t>Dokumen Formulir Permohonan &amp; Keberatan Huruf Braille (Standar &amp; Full) serta Laporan Inovasi Layanan Ramah Disabilitas PPID PKTJ Tegal</t>
         </is>
       </c>
       <c r="F94" s="16" t="inlineStr">
         <is>
-          <t>Inovasi pemenuhan sarana aksesibilitas terpadu bagi penyandang disabilitas: Formulir Permohonan Braille, Pernyataan Keberatan Braille, Audio Text-to-Speech otomatis, serta Video Panduan Bahasa Isyarat (Bisindo).</t>
+          <t>Inovasi pemenuhan sarana aksesibilitas terpadu bagi penyandang disabilitas: Formulir Permohonan Braille (Standar &amp; Full Format), Pernyataan Keberatan Braille (Standar &amp; Full Format), Audio Text-to-Speech otomatis, serta Video Panduan Bahasa Isyarat (Bisindo). Diunggah/diinput linknya melalui Menu Admin Layanan Inklusif (Braille).</t>
         </is>
       </c>
       <c r="G94" s="16" t="inlineStr">
         <is>
-          <t>FORMULIR PERMOHONAN BRAILE.pdf, PERNYATAAN KEBERATAN BRAILE.pdf, &amp; Inovasi PPID.docx (Path: AKIP PKTJ 2025\Indikator I\FORMULIR PERMOHONAN BRAILE.pdf, PERNYATAAN KEBERATAN BRAILE.pdf, &amp; Inovasi PPID.docx)</t>
+          <t>FORMULIR PERMOHONAN INFORMASI PUBLIK BRAILE.pdf, FORMULIR PERMOHONAN INFORMASI PUBLIK FULL BRAILE.pdf, PERNYATAAN KEBERATAN ATAS PERMOHONAN INFORMASI BRAILE.pdf, PERNYATAAN KEBERATAN ATAS PERMOHONAN INFORMASI FULL BRAILE.pdf, &amp; Inovasi PPID.docx (Path: AKIP PKTJ 2025\Indikator I)</t>
         </is>
       </c>
       <c r="H94" s="52" t="inlineStr">

</xml_diff>